<commit_message>
Auto update Pengadaan 2026-09-07 10:16:55
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-07).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-07).xlsx
@@ -1020,35 +1020,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1389,22 +1381,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>116218702</v>
+        <v>1301651478</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1528,13 +1520,13 @@
         <v>183</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2245544792</v>
+        <v>2236040639</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1868,13 +1860,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1305525621</v>
+        <v>1279995621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>11</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>289324708</v>
+        <v>263794708</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>11</v>
@@ -2035,25 +2027,25 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>64745634</v>
+        <v>76907682</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J44" s="9" t="n">
         <v>141024298</v>
@@ -3371,25 +3363,25 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3938</v>
+        <v>3965</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32662884242</v>
+        <v>32627850089</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>384</v>
+        <v>410</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6220243617</v>
+        <v>6185209464</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>384</v>
+        <v>410</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>5739167118.6</v>
+        <v>8733261942.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3554</v>
+        <v>3555</v>
       </c>
       <c r="J77" s="13" t="n">
         <v>26442640625</v>
@@ -5608,28 +5600,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>379426400</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>201970600</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>154581508</v>
+        <v>142419460</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>154581508</v>
+        <v>142419460</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -5642,10 +5634,10 @@
         </is>
       </c>
       <c r="M44" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N44" s="9" t="n">
-        <v>249438150</v>
+        <v>177455800</v>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1">
@@ -7560,28 +7552,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>96181052164</v>
+        <v>95965105114</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>63037623042</v>
+        <v>62893658342</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>61034481738.41</v>
+        <v>61022319690.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>28763798745</v>
+        <v>28751636697</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>9</v>
@@ -7590,10 +7582,10 @@
         <v>639056623</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>33143429122</v>
+        <v>33071446772</v>
       </c>
     </row>
   </sheetData>
@@ -8395,28 +8387,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26120170739</v>
+        <v>24671237012</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>24717574739</v>
+        <v>23268641012</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>24661273641</v>
+        <v>22864773641</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>24661273641</v>
+        <v>22864773641</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8610,13 +8602,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8841,34 +8833,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>48003814160</v>
+        <v>5652342335</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>47632716881</v>
+        <v>5281245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1997011203</v>
+        <v>906164395</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12043,34 +12035,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>181637645733</v>
+        <v>137202282996</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>139525277778</v>
+        <v>95089915041</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>67113738800.98</v>
+        <v>64131806024.98</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>134</v>
+        <v>110</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>63054805000.97</v>
+        <v>60072872224.97</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>3046617077</v>
+        <v>1955770269</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>83</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-09-07 10:40:40
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-07).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-07).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1301651478</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1520,13 +1528,13 @@
         <v>183</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2236040639</v>
+        <v>2245544792</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>11</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>263794708</v>
+        <v>289324708</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>11</v>
@@ -2027,25 +2035,25 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>76907682</v>
+        <v>64745634</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J44" s="9" t="n">
         <v>141024298</v>
@@ -3363,25 +3371,25 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3965</v>
+        <v>3938</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32627850089</v>
+        <v>32662884242</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>410</v>
+        <v>384</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6185209464</v>
+        <v>6220243617</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>410</v>
+        <v>384</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>8733261942.6</v>
+        <v>5739167118.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3555</v>
+        <v>3554</v>
       </c>
       <c r="J77" s="13" t="n">
         <v>26442640625</v>
@@ -5600,28 +5608,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>379426400</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>201970600</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>142419460</v>
+        <v>154581508</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>142419460</v>
+        <v>154581508</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -5634,10 +5642,10 @@
         </is>
       </c>
       <c r="M44" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N44" s="9" t="n">
-        <v>177455800</v>
+        <v>249438150</v>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1">
@@ -7552,28 +7560,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>95965105114</v>
+        <v>96181052164</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>62893658342</v>
+        <v>63037623042</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>61022319690.41</v>
+        <v>61034481738.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>28751636697</v>
+        <v>28763798745</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>9</v>
@@ -7582,10 +7590,10 @@
         <v>639056623</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>33071446772</v>
+        <v>33143429122</v>
       </c>
     </row>
   </sheetData>
@@ -8387,28 +8395,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26120170739</v>
+      </c>
+      <c r="E17" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>24671237012</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="F17" s="11" t="n">
-        <v>23268641012</v>
+        <v>24717574739</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>22864773641</v>
+        <v>24661273641</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>22864773641</v>
+        <v>24661273641</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8602,13 +8610,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8833,34 +8841,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>906164395</v>
+        <v>1997011203</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12035,34 +12043,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>137202282996</v>
+        <v>181637645733</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>95089915041</v>
+        <v>139525277778</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64131806024.98</v>
+        <v>67113738800.98</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>60072872224.97</v>
+        <v>63054805000.97</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1955770269</v>
+        <v>3046617077</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>83</v>

</xml_diff>